<commit_message>
try to fix player stats
</commit_message>
<xml_diff>
--- a/assets/schedule.xlsx
+++ b/assets/schedule.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sven/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sven/Develop/Sonstiges/nextjs/nordstern-app/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8A579F-3E18-774F-9C4A-DB3BC1E09FF1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6FDDD8-CAFC-9044-A5E8-465864631659}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5480" yWindow="3600" windowWidth="27840" windowHeight="16740" xr2:uid="{CC5531EC-EA4B-4C49-901F-B97AF59B9A20}"/>
   </bookViews>
@@ -523,7 +523,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="5">
-        <v>44646.833333333336</v>
+        <v>44667.791666666664</v>
       </c>
       <c r="H4" s="1"/>
     </row>
@@ -543,6 +543,12 @@
       <c r="E5" s="5">
         <v>44645.833333333336</v>
       </c>
+      <c r="F5" s="7">
+        <v>13</v>
+      </c>
+      <c r="G5" s="7">
+        <v>7</v>
+      </c>
       <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -561,6 +567,12 @@
       <c r="E6" s="5">
         <v>44646.666666666664</v>
       </c>
+      <c r="F6" s="7">
+        <v>11</v>
+      </c>
+      <c r="G6" s="7">
+        <v>10</v>
+      </c>
       <c r="H6" s="1"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -579,6 +591,12 @@
       <c r="E7" s="5">
         <v>44653.791666666664</v>
       </c>
+      <c r="F7" s="7">
+        <v>12</v>
+      </c>
+      <c r="G7" s="7">
+        <v>8</v>
+      </c>
       <c r="H7" s="1"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -597,6 +615,12 @@
       <c r="E8" s="5">
         <v>44653.770833333336</v>
       </c>
+      <c r="F8" s="7">
+        <v>15</v>
+      </c>
+      <c r="G8" s="7">
+        <v>5</v>
+      </c>
       <c r="H8" s="1"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -614,6 +638,12 @@
       </c>
       <c r="E9" s="5">
         <v>44652.833333333336</v>
+      </c>
+      <c r="F9" s="7">
+        <v>15</v>
+      </c>
+      <c r="G9" s="7">
+        <v>5</v>
       </c>
       <c r="H9" s="1"/>
     </row>
@@ -678,6 +708,12 @@
       </c>
       <c r="E12" s="5">
         <v>44660.833333333336</v>
+      </c>
+      <c r="F12" s="7">
+        <v>7</v>
+      </c>
+      <c r="G12" s="7">
+        <v>13</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>

</xml_diff>